<commit_message>
Fixes cash flows for process emissions & adds new GRAs for clean heat PTC/ITC and process emissions
</commit_message>
<xml_diff>
--- a/InputData/ctrl-settings/GRA/Government Revenue Accounting.xlsx
+++ b/InputData/ctrl-settings/GRA/Government Revenue Accounting.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\ctrl-settings\GRA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\ctrl-settings\GRA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2B31A74-FEF5-46AA-8455-B6AF2D8FAC31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA535897-C158-455B-97C1-68C21FCB72E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="698" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="25980" windowHeight="14640" tabRatio="698" firstSheet="9" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,9 @@
     <sheet name="GRA-fuelsubsidy" sheetId="14" r:id="rId10"/>
     <sheet name="GRA-CCSsubsidy" sheetId="17" r:id="rId11"/>
     <sheet name="GRA-ntnldebtinterest" sheetId="15" r:id="rId12"/>
-    <sheet name="GRA-remainder" sheetId="16" r:id="rId13"/>
+    <sheet name="GRA-indstcleanheat" sheetId="19" r:id="rId13"/>
+    <sheet name="GRA-indstprocemiss" sheetId="20" r:id="rId14"/>
+    <sheet name="GRA-remainder" sheetId="16" r:id="rId15"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -48,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="65">
   <si>
     <t>GRA Government Revenue Accounting</t>
   </si>
@@ -237,6 +239,12 @@
   </si>
   <si>
     <t>Government revenue handling is one of the design decisions a model user should make</t>
+  </si>
+  <si>
+    <t>industry clean heat subsidy</t>
+  </si>
+  <si>
+    <t>industry process emissions subsidy</t>
   </si>
 </sst>
 </file>
@@ -329,7 +337,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -348,7 +356,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -365,10 +372,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1091,6 +1094,136 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7B026F0-7193-4A6C-9CD5-22217CFA3C09}">
+  <sheetPr>
+    <tabColor theme="4" tint="-0.249977111117893"/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="34.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2">
+        <f t="array" ref="B2:B6">TRANSPOSE('Set Values Here'!B15:F15)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2011B7B9-C3B4-4A05-B3BD-95BC1D6EBEEE}">
+  <sheetPr>
+    <tabColor theme="4" tint="-0.249977111117893"/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="34.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2">
+        <f t="array" ref="B2:B6">TRANSPOSE('Set Values Here'!B15:F15)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
@@ -1364,7 +1497,7 @@
       <c r="B15">
         <v>0</v>
       </c>
-      <c r="C15" s="14">
+      <c r="C15">
         <v>5</v>
       </c>
       <c r="D15">

</xml_diff>

<commit_message>
Adds hydrogen production subsidy + accounting
</commit_message>
<xml_diff>
--- a/InputData/ctrl-settings/GRA/Government Revenue Accounting.xlsx
+++ b/InputData/ctrl-settings/GRA/Government Revenue Accounting.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\ctrl-settings\GRA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA535897-C158-455B-97C1-68C21FCB72E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFE1C15A-F679-439B-86E7-7F30F2C1AEB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="25980" windowHeight="14640" tabRatio="698" firstSheet="9" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-30" yWindow="0" windowWidth="19180" windowHeight="11260" tabRatio="698" firstSheet="11" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,8 @@
     <sheet name="GRA-ntnldebtinterest" sheetId="15" r:id="rId12"/>
     <sheet name="GRA-indstcleanheat" sheetId="19" r:id="rId13"/>
     <sheet name="GRA-indstprocemiss" sheetId="20" r:id="rId14"/>
-    <sheet name="GRA-remainder" sheetId="16" r:id="rId15"/>
+    <sheet name="GRA-hydgnprodsubs" sheetId="21" r:id="rId15"/>
+    <sheet name="GRA-remainder" sheetId="16" r:id="rId16"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -50,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="66">
   <si>
     <t>GRA Government Revenue Accounting</t>
   </si>
@@ -245,6 +246,9 @@
   </si>
   <si>
     <t>industry process emissions subsidy</t>
+  </si>
+  <si>
+    <t>hydrogen production subsidy</t>
   </si>
 </sst>
 </file>
@@ -1224,6 +1228,71 @@
 </file>
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B89476C-85AD-412F-9D0D-DC84104F348D}">
+  <sheetPr>
+    <tabColor theme="4" tint="-0.249977111117893"/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="34.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2">
+        <f t="array" ref="B2:B6">TRANSPOSE('Set Values Here'!B15:F15)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>

</xml_diff>